<commit_message>
Broaden LoadCalcChecklist keywords after a second real-project rollout test
A rollout test against a second real project (F-04-00-130 Eng. Obaidat
Villa, distinct from F12-04-233) surfaced two checklist false negatives:
"Pump Head and Flow" didn't recognize a real pump calc phrased as "Total
Head Loss," and "Sump Pit and Pump Calc" didn't recognize a Sewage
Treatment Plant as a valid alternative to a sump pit. Widened both
keyword lists; re-verified against F12-04-233 afterward with zero
regression (still exactly the same 4 findings).

The same test's remaining load-calc FAIL (no sewage-handling sizing calc
of any kind in Obaidat Villa's real calc PDF) is a genuine gap, confirmed
directly against the extracted text -- not a checklist artifact.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel_templates/LoadCalcChecklist.xlsx
+++ b/docs/excel_templates/LoadCalcChecklist.xlsx
@@ -685,7 +685,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Pump Duty Calculation|Total Dynamic Head|Pump Head</t>
+          <t>Pump Duty Calculation|Total Dynamic Head|Pump Head|Total Head Loss</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Present and complete for all 7 pumps on F12-04-233.</t>
+          <t>Present and complete for all 7 pumps on F12-04-233. Keywords widened 2026-09-28 after a second real project (F-04-00-130 Eng. Obaidat Villa, rollout-test package) had real, complete pump duty calcs that used "Total Head Loss" instead -- a checklist false negative, not a missing calc. Presence-only: still cannot verify the found calc is numerically correct.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -707,17 +707,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sump Pit Sizing</t>
+          <t>Sewage Handling Sizing</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sump Pit and Pump Calc</t>
+          <t>Sump Pit and Pump Calc, or STP Calc</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sump Pit</t>
+          <t>Sump Pit|Sewage Treatment Plant|STP</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Present and complete on F12-04-233.</t>
+          <t>Present and complete on F12-04-233 (sump pit). Widened 2026-09-28: a second real project (F-04-00-130 Eng. Obaidat Villa, rollout-test package) uses a Sewage Treatment Plant instead of a sump pit -- a legitimate alternative design choice, not a missing calc. This item now accepts either.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">

</xml_diff>